<commit_message>
Update test Excel files with new data
Refreshed forecast_result.xlsx, integrated_erp.xlsx, and integrated_transit.xlsx in test/3 with updated data for testing purposes.
</commit_message>
<xml_diff>
--- a/test/3/integrated_transit.xlsx
+++ b/test/3/integrated_transit.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="844" uniqueCount="146">
   <si>
     <t>Tw</t>
   </si>
@@ -3241,6 +3241,9 @@
       <c r="P49" t="s">
         <v>143</v>
       </c>
+      <c r="Q49" t="s">
+        <v>145</v>
+      </c>
     </row>
     <row r="50" spans="5:17">
       <c r="E50" t="s">

</xml_diff>